<commit_message>
Correct System B shading reconstruction and regenerate results
</commit_message>
<xml_diff>
--- a/results/05_STATISTICAL_INFERENCE.xlsx
+++ b/results/05_STATISTICAL_INFERENCE.xlsx
@@ -1911,13 +1911,13 @@
         <v>886</v>
       </c>
       <c r="E8">
-        <v>566.9802434772816</v>
+        <v>213.3236335839051</v>
       </c>
       <c r="F8">
-        <v>528.5119375160651</v>
+        <v>156.6193129471536</v>
       </c>
       <c r="G8">
-        <v>606.4421140612546</v>
+        <v>288.9286689509184</v>
       </c>
       <c r="H8">
         <v>7</v>
@@ -1943,13 +1943,13 @@
         <v>886</v>
       </c>
       <c r="E9">
-        <v>38.07832507510927</v>
+        <v>14.32678961791182</v>
       </c>
       <c r="F9">
-        <v>33.97759329697102</v>
+        <v>9.59341020445674</v>
       </c>
       <c r="G9">
-        <v>44.33200589869241</v>
+        <v>21.71533524924125</v>
       </c>
       <c r="H9">
         <v>7</v>
@@ -1975,13 +1975,13 @@
         <v>886</v>
       </c>
       <c r="E10">
-        <v>-7.468044783360118</v>
+        <v>-4.981520572450805</v>
       </c>
       <c r="F10">
-        <v>-8.751998905267202</v>
+        <v>-6.568153922479604</v>
       </c>
       <c r="G10">
-        <v>-6.649806675378747</v>
+        <v>-4.061783933660627</v>
       </c>
       <c r="H10">
         <v>7</v>

</xml_diff>